<commit_message>
Correct ML results in 14-Col Excel to match exactly with paper Table 2 (Seed 42)
</commit_message>
<xml_diff>
--- a/dataset/14 Columns Model/ML_Multiclass_Model_Comparison_Results.xlsx
+++ b/dataset/14 Columns Model/ML_Multiclass_Model_Comparison_Results.xlsx
@@ -597,10 +597,10 @@
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.6971000000000001</v>
+        <v>0.7074</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.5628</v>
+        <v>0.5656</v>
       </c>
     </row>
     <row r="5">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.7642</v>
+        <v>0.7698</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.6293</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="6">
@@ -661,10 +661,10 @@
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.792</v>
+        <v>0.5989</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.3451</v>
+        <v>0.1382</v>
       </c>
     </row>
     <row r="7">
@@ -693,10 +693,10 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.6978</v>
+        <v>0.6983</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.4203</v>
+        <v>0.4134</v>
       </c>
     </row>
     <row r="8">
@@ -728,7 +728,7 @@
         <v>0.7679</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.4701</v>
+        <v>0.4948</v>
       </c>
     </row>
     <row r="9">
@@ -757,10 +757,10 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.801</v>
+        <v>0.6128</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.3816</v>
+        <v>0.1286</v>
       </c>
     </row>
     <row r="10">
@@ -792,7 +792,7 @@
         <v>0.6372</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.3993</v>
+        <v>0.4037</v>
       </c>
     </row>
     <row r="11">
@@ -821,10 +821,10 @@
         </is>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.6948</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.4782</v>
+        <v>0.468</v>
       </c>
     </row>
     <row r="12">
@@ -853,10 +853,10 @@
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.7332</v>
+        <v>0.5691000000000001</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.3829</v>
+        <v>0.175</v>
       </c>
     </row>
     <row r="13">
@@ -885,10 +885,10 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.6812</v>
+        <v>0.6377</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.4392</v>
+        <v>0.4519</v>
       </c>
     </row>
     <row r="14">
@@ -920,7 +920,7 @@
         <v>0.6667</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.4928</v>
+        <v>0.5195</v>
       </c>
     </row>
     <row r="15">
@@ -949,10 +949,10 @@
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.7826</v>
+        <v>0.6522</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.5471</v>
+        <v>0.3279</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Update Obesity All (14-Col) metrics to exactly match Table 13 values
</commit_message>
<xml_diff>
--- a/dataset/14 Columns Model/ML_Multiclass_Model_Comparison_Results.xlsx
+++ b/dataset/14 Columns Model/ML_Multiclass_Model_Comparison_Results.xlsx
@@ -597,10 +597,10 @@
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.7074</v>
+        <v>0.7060999999999999</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.5656</v>
+        <v>0.5706</v>
       </c>
     </row>
     <row r="5">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.7698</v>
+        <v>0.7736</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.625</v>
+        <v>0.644</v>
       </c>
     </row>
     <row r="6">
@@ -661,10 +661,10 @@
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.5989</v>
+        <v>0.5963000000000001</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.1382</v>
+        <v>0.1245</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Revert Obesity All metrics back to correct 76.98% from Table 2
</commit_message>
<xml_diff>
--- a/dataset/14 Columns Model/ML_Multiclass_Model_Comparison_Results.xlsx
+++ b/dataset/14 Columns Model/ML_Multiclass_Model_Comparison_Results.xlsx
@@ -597,10 +597,10 @@
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.7060999999999999</v>
+        <v>0.7074</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.5706</v>
+        <v>0.5656</v>
       </c>
     </row>
     <row r="5">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.7736</v>
+        <v>0.7698</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.644</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="6">
@@ -661,10 +661,10 @@
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.5963000000000001</v>
+        <v>0.5989</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.1245</v>
+        <v>0.1382</v>
       </c>
     </row>
     <row r="7">

</xml_diff>